<commit_message>
15 - materialy zrodlowe z rundy feedbacku 2026-09-04
Nowy folder 'Warsztaty LDIT - 20260904' (Makieta + Bot.docx, Etapy_procesu.png,
notatka ze spotkania 04.09). Aktualizacja 'Prowizja liczenie.xlsx' i spisu
funkcji od Bartka. Zamyka niezacommitowane zmiany, working tree czysty.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Prowizja liczenie.xlsx
+++ b/Prowizja liczenie.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://odczarujlowcode.sharepoint.com/sites/ProjektyRaportowania/Shared Documents/LDIT - PROJEKTY/System dla instytucji szkoleniowych/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="8_{48CC61ED-0273-4E0F-895F-1D2090BAE326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1208F7D0-1C5E-4E58-BF74-1BD4B94CD11F}"/>
+  <xr:revisionPtr revIDLastSave="206" documentId="8_{48CC61ED-0273-4E0F-895F-1D2090BAE326}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A968267-84E8-450E-85AC-808D75DDF4A6}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{6870F1D1-A10A-4456-AA32-C6498B1D4F8B}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{6870F1D1-A10A-4456-AA32-C6498B1D4F8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Liczenie prowizji" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="70">
   <si>
     <t>War. Szkolenia</t>
   </si>
@@ -101,9 +101,6 @@
     <t>nadwyżka</t>
   </si>
   <si>
-    <t>całość</t>
-  </si>
-  <si>
     <t>Status per wniosek</t>
   </si>
   <si>
@@ -210,6 +207,51 @@
   </si>
   <si>
     <t>czy zakwalifikowany</t>
+  </si>
+  <si>
+    <t>całość obrotu</t>
+  </si>
+  <si>
+    <t>nadwyżka nad progiem</t>
+  </si>
+  <si>
+    <t>sty</t>
+  </si>
+  <si>
+    <t>lu</t>
+  </si>
+  <si>
+    <t>marz</t>
+  </si>
+  <si>
+    <t>koszt całk</t>
+  </si>
+  <si>
+    <t>stawka</t>
+  </si>
+  <si>
+    <t>Prowizja</t>
+  </si>
+  <si>
+    <t>Progi</t>
+  </si>
+  <si>
+    <t>&lt;2000</t>
+  </si>
+  <si>
+    <t>jednorazowo</t>
+  </si>
+  <si>
+    <t>od początku roku</t>
+  </si>
+  <si>
+    <t>&lt;6000</t>
+  </si>
+  <si>
+    <t>&gt;8000</t>
+  </si>
+  <si>
+    <t>kwie</t>
   </si>
 </sst>
 </file>
@@ -218,7 +260,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="4" x14ac:knownFonts="1">
     <font>
@@ -334,24 +376,26 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Dziesiętny" xfId="1" builtinId="3"/>
@@ -426,6 +470,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -822,7 +870,7 @@
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G5" s="2">
         <v>0.12</v>
@@ -831,7 +879,7 @@
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
       <c r="F6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G6" s="2">
         <v>0.1</v>
@@ -1144,7 +1192,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2040C4A9-1917-402E-829D-E7A01F9A7422}">
-  <dimension ref="C3:G12"/>
+  <dimension ref="C1:S12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="25.28515625" customWidth="1"/>
@@ -1153,9 +1201,39 @@
     <col min="6" max="6" width="15.5703125" customWidth="1"/>
     <col min="7" max="7" width="24.42578125" customWidth="1"/>
     <col min="8" max="8" width="16" customWidth="1"/>
+    <col min="11" max="11" width="13.85546875" customWidth="1"/>
+    <col min="12" max="12" width="23.42578125" customWidth="1"/>
+    <col min="13" max="13" width="16.42578125" customWidth="1"/>
+    <col min="14" max="14" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="3:19" x14ac:dyDescent="0.25">
+      <c r="K1" s="18" t="s">
+        <v>14</v>
+      </c>
+      <c r="L1" s="18"/>
+      <c r="M1" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="3:19" x14ac:dyDescent="0.25">
+      <c r="K2" t="s">
+        <v>60</v>
+      </c>
+      <c r="L2" t="s">
+        <v>66</v>
+      </c>
+      <c r="M2" t="s">
+        <v>61</v>
+      </c>
+      <c r="N2" t="s">
+        <v>62</v>
+      </c>
+      <c r="R2" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="3" spans="3:19" x14ac:dyDescent="0.25">
       <c r="C3" t="s">
         <v>15</v>
       </c>
@@ -1163,40 +1241,144 @@
         <v>17</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="3:7" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>57</v>
+      </c>
+      <c r="K3">
+        <v>2000</v>
+      </c>
+      <c r="L3">
+        <f>SUM(K$3:K3)</f>
+        <v>2000</v>
+      </c>
+      <c r="M3">
+        <f>0.1</f>
+        <v>0.1</v>
+      </c>
+      <c r="N3">
+        <f>K3*M3</f>
+        <v>200</v>
+      </c>
+      <c r="R3" t="s">
+        <v>64</v>
+      </c>
+      <c r="S3" s="2">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4" spans="3:19" x14ac:dyDescent="0.25">
       <c r="C4" t="s">
         <v>13</v>
       </c>
       <c r="E4" t="s">
-        <v>18</v>
+        <v>56</v>
       </c>
       <c r="G4" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="5" spans="3:7" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="J4" t="s">
+        <v>58</v>
+      </c>
+      <c r="K4">
+        <v>2000</v>
+      </c>
+      <c r="L4">
+        <f>SUM(K$3:K4)</f>
+        <v>4000</v>
+      </c>
+      <c r="M4">
+        <v>0.15</v>
+      </c>
+      <c r="N4">
+        <f t="shared" ref="N4:N5" si="0">K4*M4</f>
+        <v>300</v>
+      </c>
+      <c r="R4" t="s">
+        <v>67</v>
+      </c>
+      <c r="S4" s="2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="5" spans="3:19" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
         <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>55</v>
       </c>
       <c r="G5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="3:7" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+      <c r="J5" t="s">
+        <v>59</v>
+      </c>
+      <c r="K5">
+        <v>2000</v>
+      </c>
+      <c r="L5">
+        <f>SUM(K$3:K5)</f>
+        <v>6000</v>
+      </c>
+      <c r="M5">
+        <f t="shared" ref="M5" si="1">0.2</f>
+        <v>0.2</v>
+      </c>
+      <c r="N5">
+        <f t="shared" si="0"/>
+        <v>400</v>
+      </c>
+      <c r="R5" t="s">
+        <v>68</v>
+      </c>
+      <c r="S5" s="2">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="6" spans="3:19" x14ac:dyDescent="0.25">
       <c r="C6" t="s">
         <v>16</v>
       </c>
       <c r="E6" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="10" spans="3:7" x14ac:dyDescent="0.25">
+      <c r="J6" t="s">
+        <v>69</v>
+      </c>
+      <c r="K6">
+        <v>10000</v>
+      </c>
+      <c r="L6">
+        <f>SUM(K$3:K6)</f>
+        <v>16000</v>
+      </c>
+      <c r="M6" s="2">
+        <v>0.15</v>
+      </c>
+      <c r="N6">
+        <f>K6*M6</f>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="7" spans="3:19" x14ac:dyDescent="0.25">
+      <c r="J7" t="s">
+        <v>69</v>
+      </c>
+      <c r="K7">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="8" spans="3:19" x14ac:dyDescent="0.25">
+      <c r="R8" t="s">
+        <v>65</v>
+      </c>
+      <c r="S8" s="2">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="10" spans="3:19" x14ac:dyDescent="0.25">
       <c r="C10" s="7" t="s">
         <v>15</v>
       </c>
@@ -1207,7 +1389,7 @@
         <v>120000</v>
       </c>
     </row>
-    <row r="11" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="3:19" x14ac:dyDescent="0.25">
       <c r="C11" s="6" t="s">
         <v>13</v>
       </c>
@@ -1218,20 +1400,21 @@
         <v>12000</v>
       </c>
     </row>
-    <row r="12" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="3:19" x14ac:dyDescent="0.25">
       <c r="C12">
         <v>100000</v>
       </c>
       <c r="E12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="3">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
+    <tablePart r:id="rId4"/>
   </tableParts>
 </worksheet>
 </file>
@@ -1248,13 +1431,13 @@
   <sheetData>
     <row r="4" spans="4:6" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" t="s">
         <v>26</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>27</v>
-      </c>
-      <c r="F4" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="5" spans="4:6" x14ac:dyDescent="0.25">
@@ -1291,45 +1474,45 @@
   <sheetData>
     <row r="2" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C2" t="s">
+        <v>39</v>
+      </c>
+      <c r="N2" t="s">
         <v>40</v>
-      </c>
-      <c r="N2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="4" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" s="4"/>
       <c r="M5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="O5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="P5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="6" spans="3:16" x14ac:dyDescent="0.25">
       <c r="N6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="O6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P6">
         <v>10000</v>
@@ -1337,10 +1520,10 @@
     </row>
     <row r="7" spans="3:16" x14ac:dyDescent="0.25">
       <c r="N7" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P7">
         <v>10000</v>
@@ -1348,10 +1531,10 @@
     </row>
     <row r="8" spans="3:16" x14ac:dyDescent="0.25">
       <c r="N8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P8">
         <v>10000</v>
@@ -1359,10 +1542,10 @@
     </row>
     <row r="9" spans="3:16" x14ac:dyDescent="0.25">
       <c r="N9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="O9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P9">
         <v>10000</v>
@@ -1370,10 +1553,10 @@
     </row>
     <row r="10" spans="3:16" x14ac:dyDescent="0.25">
       <c r="N10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="O10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P10">
         <v>10000</v>
@@ -1381,10 +1564,10 @@
     </row>
     <row r="11" spans="3:16" x14ac:dyDescent="0.25">
       <c r="N11" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="O11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P11">
         <v>10000</v>
@@ -1392,13 +1575,13 @@
     </row>
     <row r="12" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C12" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="N12" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="O12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P12">
         <v>10000</v>
@@ -1406,10 +1589,10 @@
     </row>
     <row r="13" spans="3:16" x14ac:dyDescent="0.25">
       <c r="N13" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="O13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P13">
         <v>5000</v>
@@ -1417,34 +1600,34 @@
     </row>
     <row r="14" spans="3:16" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E14" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F14" t="s">
+        <v>49</v>
+      </c>
+      <c r="G14" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" t="s">
         <v>50</v>
       </c>
-      <c r="G14" t="s">
-        <v>27</v>
-      </c>
-      <c r="H14" t="s">
+      <c r="I14" t="s">
+        <v>46</v>
+      </c>
+      <c r="J14" t="s">
         <v>51</v>
       </c>
-      <c r="I14" t="s">
+      <c r="K14" t="s">
         <v>47</v>
       </c>
-      <c r="J14" t="s">
+      <c r="N14" t="s">
+        <v>37</v>
+      </c>
+      <c r="O14" t="s">
         <v>52</v>
-      </c>
-      <c r="K14" t="s">
-        <v>48</v>
-      </c>
-      <c r="N14" t="s">
-        <v>38</v>
-      </c>
-      <c r="O14" t="s">
-        <v>53</v>
       </c>
       <c r="P14">
         <v>15000</v>
@@ -1452,10 +1635,10 @@
     </row>
     <row r="15" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E15" s="2">
         <v>0.3</v>
@@ -1482,7 +1665,7 @@
         <v>90000</v>
       </c>
       <c r="N15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="O15">
         <v>0</v>
@@ -1493,10 +1676,10 @@
     </row>
     <row r="16" spans="3:16" x14ac:dyDescent="0.25">
       <c r="C16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D16" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E16" s="12">
         <v>0.3</v>
@@ -1505,7 +1688,7 @@
         <f ca="1">SUMIF(O6:P15,"x",P6:P15)</f>
         <v>90000</v>
       </c>
-      <c r="G16" s="13">
+      <c r="G16" s="14">
         <f>J16*(1-E16)</f>
         <v>62999.999999999993</v>
       </c>
@@ -1526,7 +1709,7 @@
     </row>
     <row r="17" spans="7:11" x14ac:dyDescent="0.25">
       <c r="G17" s="9">
-        <f t="shared" ref="G16:G17" si="1">J17*(1-E17)</f>
+        <f t="shared" ref="G17" si="1">J17*(1-E17)</f>
         <v>0</v>
       </c>
       <c r="H17" s="9"/>
@@ -1740,15 +1923,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="5c808c61-7593-4213-a548-41cfd5ff245d">
@@ -1759,14 +1933,49 @@
 </p:properties>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CC1ED6F-C5AD-400A-A16E-9E88577553B2}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8CC1ED6F-C5AD-400A-A16E-9E88577553B2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="5c808c61-7593-4213-a548-41cfd5ff245d"/>
+    <ds:schemaRef ds:uri="ba0ed539-3bb3-4a9d-81be-d9892850de1a"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{180443C1-DD47-4266-AD1D-F30158F609D4}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6449C99F-30EA-4481-A349-73DC2E65978E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="5c808c61-7593-4213-a548-41cfd5ff245d"/>
+    <ds:schemaRef ds:uri="ba0ed539-3bb3-4a9d-81be-d9892850de1a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6449C99F-30EA-4481-A349-73DC2E65978E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{180443C1-DD47-4266-AD1D-F30158F609D4}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>